<commit_message>
Update sales analysis dashboard
</commit_message>
<xml_diff>
--- a/sales_data_analysis.xlsx
+++ b/sales_data_analysis.xlsx
@@ -8,19 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vaish\Projects\sales-data-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{31A918A8-6A72-415D-93E6-341E1DD9C078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{07586C60-2BBC-4789-B7A6-5E49E0F60103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="17280" windowHeight="8880" xr2:uid="{92616B37-70BB-49F2-B3DA-95AA46808868}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{92616B37-70BB-49F2-B3DA-95AA46808868}"/>
   </bookViews>
   <sheets>
     <sheet name="sales" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="28">
   <si>
     <t>OrderID</t>
   </si>
@@ -78,12 +90,42 @@
   <si>
     <t>Phone</t>
   </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>Total Revenue</t>
+  </si>
+  <si>
+    <t>SALES PERFORMANCE DASHBOARD</t>
+  </si>
+  <si>
+    <t>Total Profit</t>
+  </si>
+  <si>
+    <t>Total Units Sold</t>
+  </si>
+  <si>
+    <t>Total Orders</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Profit Margin</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+  </numFmts>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,8 +260,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -399,6 +454,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -560,9 +621,20 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -608,7 +680,17 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -619,6 +701,2929 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Revenue by Product</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.15739904339368746"/>
+          <c:y val="0.18198520639465518"/>
+          <c:w val="0.89655796150481193"/>
+          <c:h val="0.72088764946048411"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>sales!$M$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>sales!$L$2:$L$6</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Keyboard</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Mouse</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>sales!$M$2:$M$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>275000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>120000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>60000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18400</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8B86-4482-B473-7793A610E7A6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1212021519"/>
+        <c:axId val="1167203695"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1212021519"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1167203695"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1167203695"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1212021519"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Monthly</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Revenue Trend</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>sales!$Q$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>sales!$P$2:$P$4</c:f>
+              <c:numCache>
+                <c:formatCode>mmm\-yy</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>46023</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46054</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46082</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>sales!$Q$2:$Q$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>142500</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>152000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>192400</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-7B88-4CD9-BCC0-9D3150D7694A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1310695983"/>
+        <c:axId val="1167198895"/>
+      </c:barChart>
+      <c:dateAx>
+        <c:axId val="1310695983"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="mmm\-yy" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1167198895"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+        <c:baseTimeUnit val="months"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="1167198895"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1310695983"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>Profit by Product</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>sales!$N$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profit</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>sales!$L$2:$L$6</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Keyboard</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Mouse</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>sales!$N$2:$N$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>65000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6300</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4E8A-4638-AC5A-316039DB9AD6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="120491024"/>
+        <c:axId val="117742032"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="120491024"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="117742032"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="117742032"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="120491024"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>350520</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>731520</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6254CD0-8002-4529-AF75-7978B83D023F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C84428C7-AFEC-4D15-BA5C-782C76A6B67D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A56D5773-9722-4183-9FF8-67AD8940B39D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EF8FF7E9-DC6B-4816-836C-F969A0D354A3}" name="SalesTable" displayName="SalesTable" ref="A1:J13" totalsRowShown="0">
+  <autoFilter ref="A1:J13" xr:uid="{EF8FF7E9-DC6B-4816-836C-F969A0D354A3}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{B813CBED-B2A1-485D-A9F3-19916F110979}" name="OrderID"/>
+    <tableColumn id="2" xr3:uid="{C702EE33-B601-492C-929E-07802CE881E4}" name="OrderDate" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{7844D52A-65F2-46C4-BA67-AC6FAB74254D}" name="Region"/>
+    <tableColumn id="4" xr3:uid="{7A810535-BC3D-460D-A16C-13A5280FABC1}" name="Product"/>
+    <tableColumn id="5" xr3:uid="{4765BBF2-953A-4B15-9D07-EF1713F59DF9}" name="Category"/>
+    <tableColumn id="6" xr3:uid="{B89D99CD-DD77-4084-A629-B4F9345276AC}" name="Quantity"/>
+    <tableColumn id="7" xr3:uid="{F858AF74-A3D2-4D2A-96DD-9D009333BE70}" name="UnitPrice"/>
+    <tableColumn id="8" xr3:uid="{B55093B0-9711-4A65-9944-92239960F417}" name="UnitCost"/>
+    <tableColumn id="9" xr3:uid="{97622146-75CC-406A-A506-B36D5DEFC1FD}" name="Revenue" dataDxfId="1">
+      <calculatedColumnFormula>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{C40800B7-12C9-46A6-B2FB-5B8519EF99F0}" name="Profit" dataDxfId="0">
+      <calculatedColumnFormula>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -918,10 +3923,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A30C419-FC11-4DE0-AC84-65009819CC5F}">
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:T13"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" customWidth="1"/>
+    <col min="19" max="19" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -946,8 +3961,36 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+      <c r="S1" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="5">
+        <f>125500/486900</f>
+        <v>0.25775313205997125</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -972,8 +4015,34 @@
       <c r="H2">
         <v>42000</v>
       </c>
+      <c r="I2">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>110000</v>
+      </c>
+      <c r="J2">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>26000</v>
+      </c>
+      <c r="L2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2">
+        <f>SUMIF($D$2:$D$13,L2,$I$2:$I$13)</f>
+        <v>275000</v>
+      </c>
+      <c r="N2">
+        <f>SUMIF($D$2:$D$13,L2,$J$2:$J$13)</f>
+        <v>65000</v>
+      </c>
+      <c r="P2" s="4">
+        <v>46023</v>
+      </c>
+      <c r="Q2">
+        <f>SUMIFS($I$2:$I$13,$B$2:$B$13,"&gt;="&amp;DATE(2026,1,1),$B$2:$B$13,"&lt;"&amp;DATE(2026,2,1))</f>
+        <v>142500</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -998,8 +4067,34 @@
       <c r="H3">
         <v>400</v>
       </c>
+      <c r="I3">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>4000</v>
+      </c>
+      <c r="J3">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>2000</v>
+      </c>
+      <c r="L3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3">
+        <f>SUMIF($D$2:$D$13,L3,$I$2:$I$13)</f>
+        <v>120000</v>
+      </c>
+      <c r="N3">
+        <f>SUMIF($D$2:$D$13,L3,$J$2:$J$13)</f>
+        <v>30000</v>
+      </c>
+      <c r="P3" s="4">
+        <v>46054</v>
+      </c>
+      <c r="Q3">
+        <f>SUMIFS($I$2:$I$13,$B$2:$B$13,"&gt;="&amp;DATE(2026,2,1),$B$2:$B$13,"&lt;"&amp;DATE(2026,3,1))</f>
+        <v>152000</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1024,8 +4119,34 @@
       <c r="H4">
         <v>800</v>
       </c>
+      <c r="I4">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>4500</v>
+      </c>
+      <c r="J4">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>2100</v>
+      </c>
+      <c r="L4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4">
+        <f>SUMIF($D$2:$D$13,L4,$I$2:$I$13)</f>
+        <v>60000</v>
+      </c>
+      <c r="N4">
+        <f>SUMIF($D$2:$D$13,L4,$J$2:$J$13)</f>
+        <v>15000</v>
+      </c>
+      <c r="P4" s="4">
+        <v>46082</v>
+      </c>
+      <c r="Q4">
+        <f>SUMIFS($I$2:$I$13,$B$2:$B$13,"&gt;="&amp;DATE(2026,3,1),$B$2:$B$13,"&lt;"&amp;DATE(2026,4,1))</f>
+        <v>192400</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -1050,8 +4171,27 @@
       <c r="H5">
         <v>9000</v>
       </c>
+      <c r="I5">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>24000</v>
+      </c>
+      <c r="J5">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>6000</v>
+      </c>
+      <c r="L5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M5">
+        <f>SUMIF($D$2:$D$13,L5,$I$2:$I$13)</f>
+        <v>13500</v>
+      </c>
+      <c r="N5">
+        <f>SUMIF($D$2:$D$13,L5,$J$2:$J$13)</f>
+        <v>6300</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -1076,8 +4216,27 @@
       <c r="H6">
         <v>15000</v>
       </c>
+      <c r="I6">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>80000</v>
+      </c>
+      <c r="J6">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>20000</v>
+      </c>
+      <c r="L6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M6">
+        <f>SUMIF($D$2:$D$13,L6,$I$2:$I$13)</f>
+        <v>18400</v>
+      </c>
+      <c r="N6">
+        <f>SUMIF($D$2:$D$13,L6,$J$2:$J$13)</f>
+        <v>9200</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -1102,8 +4261,16 @@
       <c r="H7">
         <v>42000</v>
       </c>
+      <c r="I7">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>55000</v>
+      </c>
+      <c r="J7">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>13000</v>
+      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1128,8 +4295,16 @@
       <c r="H8">
         <v>400</v>
       </c>
+      <c r="I8">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>8000</v>
+      </c>
+      <c r="J8">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>4000</v>
+      </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1154,8 +4329,16 @@
       <c r="H9">
         <v>800</v>
       </c>
+      <c r="I9">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>9000</v>
+      </c>
+      <c r="J9">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>4200</v>
+      </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1180,8 +4363,16 @@
       <c r="H10">
         <v>9000</v>
       </c>
+      <c r="I10">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>36000</v>
+      </c>
+      <c r="J10">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>9000</v>
+      </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1206,8 +4397,16 @@
       <c r="H11">
         <v>15000</v>
       </c>
+      <c r="I11">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>40000</v>
+      </c>
+      <c r="J11">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>10000</v>
+      </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20">
       <c r="A12">
         <v>1011</v>
       </c>
@@ -1232,8 +4431,16 @@
       <c r="H12">
         <v>42000</v>
       </c>
+      <c r="I12">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>110000</v>
+      </c>
+      <c r="J12">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>26000</v>
+      </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20">
       <c r="A13">
         <v>1012</v>
       </c>
@@ -1257,9 +4464,88 @@
       </c>
       <c r="H13">
         <v>400</v>
+      </c>
+      <c r="I13">
+        <f>SalesTable[[#This Row],[Quantity]]*SalesTable[[#This Row],[UnitPrice]]</f>
+        <v>6400</v>
+      </c>
+      <c r="J13">
+        <f>SalesTable[[#This Row],[Quantity]]*(SalesTable[[#This Row],[UnitPrice]]-SalesTable[[#This Row],[UnitCost]])</f>
+        <v>3200</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{617BEE86-485B-4674-85BC-71ED9CC5820C}">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="23.4" customHeight="1">
+      <c r="A1" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="3">
+        <f>SUM(SalesTable[Revenue])</f>
+        <v>486900</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="3">
+        <f>SUM(SalesTable[Profit])</f>
+        <v>125500</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="2">
+        <f>SUM(SalesTable[Quantity])</f>
+        <v>48</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="2">
+        <f>COUNTA(SalesTable[OrderID])</f>
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>